<commit_message>
Updated classifier to support simple, medium, complex categories
</commit_message>
<xml_diff>
--- a/srs_data_sample.xlsx
+++ b/srs_data_sample.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://brillioonline-my.sharepoint.com/personal/nagineni_sireesha_brillio_com/Documents/Documents/mcp_cve_new/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://brillioonline-my.sharepoint.com/personal/nagineni_sireesha_brillio_com/Documents/Documents/streamlit-remediation-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{AD689765-A2E6-4F0F-B39D-56B89017E083}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FFD4E18-84FE-4E9E-A4A8-B667F1A968FE}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="8_{AD689765-A2E6-4F0F-B39D-56B89017E083}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{790641BA-4534-467B-A104-FDA73F23AE3F}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D4480F6B-9C63-49C4-94D0-59B3827A0F1B}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$BF$8</definedName>
     <definedName name="_Toc216332146" localSheetId="0">Sheet1!$C$8</definedName>
     <definedName name="_Toc216332154" localSheetId="0">Sheet1!$C$2</definedName>
   </definedNames>
@@ -578,6 +579,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -897,11 +902,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABF2DD4F-3D5F-47E5-A976-C28A69E3B1CA}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:BF10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="36.7265625" customWidth="1"/>
     <col min="3" max="3" width="33.26953125" customWidth="1"/>
+    <col min="4" max="4" width="31.08984375" customWidth="1"/>
     <col min="19" max="19" width="21.453125" customWidth="1"/>
     <col min="26" max="26" width="34.6328125" customWidth="1"/>
     <col min="27" max="27" width="25.54296875" customWidth="1"/>
@@ -1085,7 +1092,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:58" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:58" ht="409.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>64</v>
       </c>
@@ -1195,7 +1202,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="3" spans="1:58" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:58" ht="409.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>80</v>
       </c>
@@ -1305,7 +1312,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="4" spans="1:58" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:58" ht="409.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>85</v>
       </c>
@@ -1418,7 +1425,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="5" spans="1:58" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:58" ht="409.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>94</v>
       </c>
@@ -1531,7 +1538,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="6" spans="1:58" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:58" ht="409.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>101</v>
       </c>
@@ -1775,7 +1782,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="8" spans="1:58" ht="362.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:58" ht="362.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>130</v>
       </c>
@@ -1907,6 +1914,13 @@
       <c r="S10" s="1"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:BF8" xr:uid="{ABF2DD4F-3D5F-47E5-A976-C28A69E3B1CA}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="CVE-2025-1153"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <hyperlinks>
     <hyperlink ref="Z3" r:id="rId1" xr:uid="{E166C79F-C7FA-4974-B736-7EAA1A8DE8E3}"/>
     <hyperlink ref="Z7" r:id="rId2" xr:uid="{0854D9F8-E6D4-4B2C-B26E-D28DE11F56BD}"/>

</xml_diff>